<commit_message>
Baek, Hyeongjun KRW 매칭 추가
</commit_message>
<xml_diff>
--- a/Diplat_Korea_2026_Mar.xlsx
+++ b/Diplat_Korea_2026_Mar.xlsx
@@ -16,10 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="#,##0.##"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="#,##0.##"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -85,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,11 +106,55 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -119,7 +162,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -128,13 +171,13 @@
     <xf numFmtId="1" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,7 +186,7 @@
     <xf numFmtId="1" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -156,7 +199,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,6 +228,23 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -637,7 +697,7 @@
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="27" t="n">
         <v>46087</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -663,16 +723,16 @@
           <t>WICKED3</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="28" t="n">
         <v>123</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="28" t="n">
         <v>246</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="28" t="n">
         <v>246</v>
       </c>
       <c r="K3" s="7" t="n">
@@ -683,7 +743,7 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="29" t="n">
         <v>46089</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -709,16 +769,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="30" t="n">
         <v>134</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="I4" s="30" t="n">
         <v>134</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="30" t="n">
         <v>134</v>
       </c>
       <c r="K4" s="12" t="n">
@@ -729,7 +789,7 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="27" t="n">
         <v>46089</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -755,16 +815,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="28" t="n">
         <v>187</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="28" t="n">
         <v>748</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="28" t="n">
         <v>748</v>
       </c>
       <c r="K5" s="7" t="n">
@@ -775,7 +835,7 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="29" t="n">
         <v>46090</v>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -801,16 +861,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="30" t="n">
         <v>93</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="30" t="n">
         <v>186</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="30" t="n">
         <v>186</v>
       </c>
       <c r="K6" s="12" t="n">
@@ -821,7 +881,7 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="27" t="n">
         <v>46090</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -847,16 +907,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="28" t="n">
         <v>116</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="28" t="n">
         <v>232</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="28" t="n">
         <v>232</v>
       </c>
       <c r="K7" s="7" t="n">
@@ -867,7 +927,7 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="29" t="n">
         <v>46090</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -893,16 +953,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="30" t="n">
         <v>122</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="30" t="n">
         <v>244</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="30" t="n">
         <v>244</v>
       </c>
       <c r="K8" s="12" t="n">
@@ -913,7 +973,7 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="27" t="n">
         <v>46091</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -939,16 +999,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="28" t="n">
         <v>122</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="28" t="n">
         <v>244</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="J9" s="28" t="n">
         <v>244</v>
       </c>
       <c r="K9" s="7" t="n">
@@ -959,7 +1019,7 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="29" t="n">
         <v>46092</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -985,16 +1045,16 @@
           <t>CURSEDCHIL</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="30" t="n">
         <v>159</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="30" t="n">
         <v>318</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="30" t="n">
         <v>318</v>
       </c>
       <c r="K10" s="12" t="n">
@@ -1005,7 +1065,7 @@
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="27" t="n">
         <v>46092</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1031,16 +1091,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="28" t="n">
         <v>93</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="28" t="n">
         <v>186</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="J11" s="28" t="n">
         <v>186</v>
       </c>
       <c r="K11" s="7" t="n">
@@ -1051,7 +1111,7 @@
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="29" t="n">
         <v>46092</v>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -1077,16 +1137,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="30" t="n">
         <v>93</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="30" t="n">
         <v>186</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="30" t="n">
         <v>186</v>
       </c>
       <c r="K12" s="12" t="n">
@@ -1097,7 +1157,7 @@
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="27" t="n">
         <v>46092</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1123,16 +1183,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="28" t="n">
         <v>134</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="28" t="n">
         <v>536</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="J13" s="28" t="n">
         <v>536</v>
       </c>
       <c r="K13" s="7" t="n">
@@ -1143,7 +1203,7 @@
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="29" t="n">
         <v>46093</v>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1169,16 +1229,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="30" t="n">
         <v>134</v>
       </c>
-      <c r="I14" s="11" t="n">
+      <c r="I14" s="30" t="n">
         <v>536</v>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="J14" s="30" t="n">
         <v>536</v>
       </c>
       <c r="K14" s="12" t="n">
@@ -1189,7 +1249,7 @@
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="27" t="n">
         <v>46096</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1215,16 +1275,16 @@
           <t>WICKED3</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="28" t="n">
         <v>163</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="28" t="n">
         <v>326</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="28" t="n">
         <v>326</v>
       </c>
       <c r="K15" s="7" t="n">
@@ -1235,7 +1295,7 @@
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="29" t="n">
         <v>46096</v>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -1261,16 +1321,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H16" s="30" t="n">
         <v>93</v>
       </c>
-      <c r="I16" s="11" t="n">
+      <c r="I16" s="30" t="n">
         <v>186</v>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="J16" s="30" t="n">
         <v>186</v>
       </c>
       <c r="K16" s="12" t="n">
@@ -1281,7 +1341,7 @@
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="27" t="n">
         <v>46098</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1307,16 +1367,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H17" s="28" t="n">
         <v>233</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I17" s="28" t="n">
         <v>466</v>
       </c>
-      <c r="J17" s="6" t="n">
+      <c r="J17" s="28" t="n">
         <v>466</v>
       </c>
       <c r="K17" s="7" t="n">
@@ -1327,7 +1387,7 @@
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="29" t="n">
         <v>46098</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -1353,16 +1413,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
+      <c r="G18" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H18" s="11" t="n">
+      <c r="H18" s="30" t="n">
         <v>113</v>
       </c>
-      <c r="I18" s="11" t="n">
+      <c r="I18" s="30" t="n">
         <v>226</v>
       </c>
-      <c r="J18" s="11" t="n">
+      <c r="J18" s="30" t="n">
         <v>226</v>
       </c>
       <c r="K18" s="12" t="n">
@@ -1373,7 +1433,7 @@
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="27" t="n">
         <v>46098</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1399,16 +1459,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="28" t="n">
         <v>116</v>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I19" s="28" t="n">
         <v>232</v>
       </c>
-      <c r="J19" s="6" t="n">
+      <c r="J19" s="28" t="n">
         <v>232</v>
       </c>
       <c r="K19" s="7" t="n">
@@ -1419,7 +1479,7 @@
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="8" t="n">
+      <c r="A20" s="29" t="n">
         <v>46098</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1445,16 +1505,16 @@
           <t>CHICAGO</t>
         </is>
       </c>
-      <c r="G20" s="11" t="n">
+      <c r="G20" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="11" t="n">
+      <c r="H20" s="30" t="n">
         <v>208</v>
       </c>
-      <c r="I20" s="11" t="n">
+      <c r="I20" s="30" t="n">
         <v>416</v>
       </c>
-      <c r="J20" s="11" t="n">
+      <c r="J20" s="30" t="n">
         <v>416</v>
       </c>
       <c r="K20" s="12" t="n">
@@ -1465,7 +1525,7 @@
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="27" t="n">
         <v>46098</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1491,16 +1551,16 @@
           <t>MJMUSICAL3</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H21" s="28" t="n">
         <v>197</v>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="I21" s="28" t="n">
         <v>394</v>
       </c>
-      <c r="J21" s="6" t="n">
+      <c r="J21" s="28" t="n">
         <v>394</v>
       </c>
       <c r="K21" s="7" t="n">
@@ -1511,7 +1571,7 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="29" t="n">
         <v>46101</v>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1537,16 +1597,16 @@
           <t>HAMILTON3</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
+      <c r="G22" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H22" s="11" t="n">
+      <c r="H22" s="30" t="n">
         <v>347.7</v>
       </c>
-      <c r="I22" s="11" t="n">
+      <c r="I22" s="30" t="n">
         <v>695.4</v>
       </c>
-      <c r="J22" s="11" t="n">
+      <c r="J22" s="30" t="n">
         <v>695.4</v>
       </c>
       <c r="K22" s="12" t="n">
@@ -1557,7 +1617,7 @@
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="27" t="n">
         <v>46102</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1583,16 +1643,16 @@
           <t>LIONKING3</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="28" t="n">
         <v>277</v>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="I23" s="28" t="n">
         <v>554</v>
       </c>
-      <c r="J23" s="6" t="n">
+      <c r="J23" s="28" t="n">
         <v>554</v>
       </c>
       <c r="K23" s="7" t="n">
@@ -1603,7 +1663,7 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="8" t="n">
+      <c r="A24" s="29" t="n">
         <v>46103</v>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1629,16 +1689,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
+      <c r="G24" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="H24" s="11" t="n">
+      <c r="H24" s="30" t="n">
         <v>197</v>
       </c>
-      <c r="I24" s="11" t="n">
+      <c r="I24" s="30" t="n">
         <v>591</v>
       </c>
-      <c r="J24" s="11" t="n">
+      <c r="J24" s="30" t="n">
         <v>591</v>
       </c>
       <c r="K24" s="12" t="n">
@@ -1649,7 +1709,7 @@
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="27" t="n">
         <v>46103</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1675,16 +1735,16 @@
           <t>WICKED3</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G25" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="6" t="n">
+      <c r="H25" s="28" t="n">
         <v>123</v>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="I25" s="28" t="n">
         <v>369</v>
       </c>
-      <c r="J25" s="6" t="n">
+      <c r="J25" s="28" t="n">
         <v>369</v>
       </c>
       <c r="K25" s="7" t="n">
@@ -1695,7 +1755,7 @@
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="29" t="n">
         <v>46103</v>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1721,16 +1781,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G26" s="11" t="n">
+      <c r="G26" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="11" t="n">
+      <c r="H26" s="30" t="n">
         <v>105</v>
       </c>
-      <c r="I26" s="11" t="n">
+      <c r="I26" s="30" t="n">
         <v>210</v>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="J26" s="30" t="n">
         <v>210</v>
       </c>
       <c r="K26" s="12" t="n">
@@ -1741,7 +1801,7 @@
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="27" t="n">
         <v>46105</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1767,16 +1827,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="G27" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H27" s="6" t="n">
+      <c r="H27" s="28" t="n">
         <v>93</v>
       </c>
-      <c r="I27" s="6" t="n">
+      <c r="I27" s="28" t="n">
         <v>186</v>
       </c>
-      <c r="J27" s="6" t="n">
+      <c r="J27" s="28" t="n">
         <v>186</v>
       </c>
       <c r="K27" s="7" t="n">
@@ -1787,7 +1847,7 @@
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="29" t="n">
         <v>46106</v>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1813,16 +1873,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
+      <c r="G28" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="11" t="n">
+      <c r="H28" s="30" t="n">
         <v>197</v>
       </c>
-      <c r="I28" s="11" t="n">
+      <c r="I28" s="30" t="n">
         <v>197</v>
       </c>
-      <c r="J28" s="11" t="n">
+      <c r="J28" s="30" t="n">
         <v>197</v>
       </c>
       <c r="K28" s="12" t="n">
@@ -1833,7 +1893,7 @@
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="27" t="n">
         <v>46107</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1859,16 +1919,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G29" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="6" t="n">
+      <c r="H29" s="28" t="n">
         <v>122</v>
       </c>
-      <c r="I29" s="6" t="n">
+      <c r="I29" s="28" t="n">
         <v>244</v>
       </c>
-      <c r="J29" s="6" t="n">
+      <c r="J29" s="28" t="n">
         <v>244</v>
       </c>
       <c r="K29" s="7" t="n">
@@ -1879,7 +1939,7 @@
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="8" t="n">
+      <c r="A30" s="29" t="n">
         <v>46109</v>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1905,16 +1965,16 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
+      <c r="G30" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H30" s="11" t="n">
+      <c r="H30" s="30" t="n">
         <v>134</v>
       </c>
-      <c r="I30" s="11" t="n">
+      <c r="I30" s="30" t="n">
         <v>268</v>
       </c>
-      <c r="J30" s="11" t="n">
+      <c r="J30" s="30" t="n">
         <v>268</v>
       </c>
       <c r="K30" s="12" t="n">
@@ -1925,7 +1985,7 @@
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="27" t="n">
         <v>46112</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1951,20 +2011,24 @@
           <t>ALADDIN</t>
         </is>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G31" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H31" s="6" t="n">
+      <c r="H31" s="28" t="n">
         <v>187</v>
       </c>
-      <c r="I31" s="6" t="n">
+      <c r="I31" s="28" t="n">
         <v>374</v>
       </c>
-      <c r="J31" s="6" t="n">
+      <c r="J31" s="28" t="n">
         <v>374</v>
       </c>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="13" t="n"/>
+      <c r="K31" s="13" t="n">
+        <v>679214</v>
+      </c>
+      <c r="L31" s="13" t="n">
+        <v>665766</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="14" t="n"/>
@@ -1977,16 +2041,16 @@
       <c r="D32" s="14" t="n"/>
       <c r="E32" s="14" t="n"/>
       <c r="F32" s="14" t="n"/>
-      <c r="G32" s="16">
+      <c r="G32" s="31">
         <f>SUM(G3:G31)</f>
         <v/>
       </c>
       <c r="H32" s="14" t="n"/>
-      <c r="I32" s="16">
+      <c r="I32" s="31">
         <f>SUM(I3:I31)</f>
         <v/>
       </c>
-      <c r="J32" s="16">
+      <c r="J32" s="31">
         <f>SUM(J3:J31)</f>
         <v/>
       </c>
@@ -2001,6 +2065,14 @@
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="18" t="inlineStr"/>
+      <c r="B33" s="32" t="n"/>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="32" t="n"/>
+      <c r="F33" s="32" t="n"/>
+      <c r="G33" s="32" t="n"/>
+      <c r="H33" s="32" t="n"/>
+      <c r="I33" s="33" t="n"/>
       <c r="J33" s="19" t="n"/>
       <c r="K33" s="20" t="n"/>
       <c r="L33" s="20" t="n"/>
@@ -2011,6 +2083,13 @@
           <t>KRW거래금액 ÷ TotalSale(USD) = 환율</t>
         </is>
       </c>
+      <c r="B34" s="32" t="n"/>
+      <c r="C34" s="32" t="n"/>
+      <c r="D34" s="32" t="n"/>
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="32" t="n"/>
+      <c r="G34" s="32" t="n"/>
+      <c r="H34" s="33" t="n"/>
       <c r="I34" s="21" t="inlineStr">
         <is>
           <t>환율</t>
@@ -2028,6 +2107,13 @@
           <t>KRW정산금액 - (TotalSale × 환율) = 차액 (PG 수수료)</t>
         </is>
       </c>
+      <c r="B35" s="32" t="n"/>
+      <c r="C35" s="32" t="n"/>
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="32" t="n"/>
+      <c r="F35" s="32" t="n"/>
+      <c r="G35" s="32" t="n"/>
+      <c r="H35" s="33" t="n"/>
       <c r="I35" s="21" t="inlineStr">
         <is>
           <t>차액</t>
@@ -2045,6 +2131,13 @@
           <t>광고비</t>
         </is>
       </c>
+      <c r="B36" s="32" t="n"/>
+      <c r="C36" s="32" t="n"/>
+      <c r="D36" s="32" t="n"/>
+      <c r="E36" s="32" t="n"/>
+      <c r="F36" s="32" t="n"/>
+      <c r="G36" s="32" t="n"/>
+      <c r="H36" s="33" t="n"/>
       <c r="I36" s="21" t="inlineStr">
         <is>
           <t>광고비</t>
@@ -2060,6 +2153,13 @@
           <t>최종 정산금 = KRW정산금액 - 광고비</t>
         </is>
       </c>
+      <c r="B37" s="32" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="33" t="n"/>
       <c r="I37" s="24" t="inlineStr">
         <is>
           <t>최종 정산금</t>

</xml_diff>